<commit_message>
Freeze cleaned Q5 results and add figures
</commit_message>
<xml_diff>
--- a/projects/2025-cumcm-a-smoke-screen/results/frozen/result3.xlsx
+++ b/projects/2025-cumcm-a-smoke-screen/results/frozen/result3.xlsx
@@ -627,41 +627,9 @@
           <t>FY1</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>179.0525351904915</v>
-      </c>
-      <c r="C4" t="n">
-        <v>105.2918637512128</v>
-      </c>
       <c r="D4" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E4" t="n">
-        <v>16739.85277989637</v>
-      </c>
-      <c r="F4" t="n">
-        <v>17.53259592494768</v>
-      </c>
-      <c r="G4" t="n">
-        <v>1800</v>
-      </c>
-      <c r="H4" t="n">
-        <v>16465.92704250501</v>
-      </c>
-      <c r="I4" t="n">
-        <v>22.06274907354215</v>
-      </c>
-      <c r="J4" t="n">
-        <v>1766.826530392486</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -1057,41 +1025,9 @@
           <t>FY5</t>
         </is>
       </c>
-      <c r="B15" t="n">
-        <v>92.97298263785056</v>
-      </c>
-      <c r="C15" t="n">
-        <v>134.5297763233862</v>
-      </c>
       <c r="D15" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="E15" t="n">
-        <v>12891.99149666184</v>
-      </c>
-      <c r="F15" t="n">
-        <v>79.68805714965811</v>
-      </c>
-      <c r="G15" t="n">
-        <v>1300</v>
-      </c>
-      <c r="H15" t="n">
-        <v>12835.15529549102</v>
-      </c>
-      <c r="I15" t="n">
-        <v>1174.060862396664</v>
-      </c>
-      <c r="J15" t="n">
-        <v>974.8680535722999</v>
-      </c>
-      <c r="K15" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>M1</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -1099,40 +1035,8 @@
           <t>FY5</t>
         </is>
       </c>
-      <c r="B16" t="n">
-        <v>92.97298263785056</v>
-      </c>
-      <c r="C16" t="n">
-        <v>134.5297763233862</v>
-      </c>
       <c r="D16" s="3" t="n">
         <v>3</v>
-      </c>
-      <c r="E16" t="n">
-        <v>12812.38932586603</v>
-      </c>
-      <c r="F16" t="n">
-        <v>1612.416303637314</v>
-      </c>
-      <c r="G16" t="n">
-        <v>1300</v>
-      </c>
-      <c r="H16" t="n">
-        <v>12801.55030376294</v>
-      </c>
-      <c r="I16" t="n">
-        <v>1821.120101229921</v>
-      </c>
-      <c r="J16" t="n">
-        <v>1288.175310045826</v>
-      </c>
-      <c r="K16" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>M1</t>
-        </is>
       </c>
     </row>
     <row r="18" ht="60" customHeight="1" s="4">

</xml_diff>